<commit_message>
ajustes nos titulos das colunas
</commit_message>
<xml_diff>
--- a/Safe Child LLM/Chat GPT - Safe Child LLM.xlsx
+++ b/Safe Child LLM/Chat GPT - Safe Child LLM.xlsx
@@ -25,16 +25,16 @@
     <t xml:space="preserve">Prompt</t>
   </si>
   <si>
-    <t xml:space="preserve">Ana, adolescente cis, 15 anos</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Felipe, adolescente cis, 16 anos</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Geovana, adolescente trans, 14 anos</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Italo, adolescente trans, 15 anos</t>
+    <t xml:space="preserve">Ana, garota cis, 15 anos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Felipe, garoto cis, 16 anos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Geovana, garota trans, 14 anos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Italo, garoto trans, 15 anos</t>
   </si>
   <si>
     <t xml:space="preserve">Ariel, adolescente não binário, 16 anos</t>
@@ -3257,7 +3257,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -3277,6 +3277,13 @@
     </font>
     <font>
       <sz val="10"/>
+      <name val="Arial"/>
+      <family val="0"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="12"/>
+      <color rgb="FFFFFFFF"/>
       <name val="Arial"/>
       <family val="0"/>
     </font>
@@ -3344,24 +3351,28 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -3558,1051 +3569,1051 @@
   <dimension ref="A1:Z51"/>
   <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="27"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="32.25"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="32.88"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="37.63"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="34.63"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="42"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="27"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="32.25"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="32.88"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="37.63"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="34.63"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="42"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="2"/>
-      <c r="H1" s="2"/>
-      <c r="I1" s="2"/>
-      <c r="J1" s="2"/>
-      <c r="K1" s="2"/>
-      <c r="L1" s="2"/>
-      <c r="M1" s="2"/>
-      <c r="N1" s="2"/>
-      <c r="O1" s="2"/>
-      <c r="P1" s="2"/>
-      <c r="Q1" s="2"/>
-      <c r="R1" s="2"/>
-      <c r="S1" s="2"/>
-      <c r="T1" s="2"/>
-      <c r="U1" s="2"/>
-      <c r="V1" s="2"/>
-      <c r="W1" s="2"/>
-      <c r="X1" s="2"/>
-      <c r="Y1" s="2"/>
-      <c r="Z1" s="2"/>
+      <c r="G1" s="4"/>
+      <c r="H1" s="4"/>
+      <c r="I1" s="4"/>
+      <c r="J1" s="4"/>
+      <c r="K1" s="4"/>
+      <c r="L1" s="4"/>
+      <c r="M1" s="4"/>
+      <c r="N1" s="4"/>
+      <c r="O1" s="4"/>
+      <c r="P1" s="4"/>
+      <c r="Q1" s="4"/>
+      <c r="R1" s="4"/>
+      <c r="S1" s="4"/>
+      <c r="T1" s="4"/>
+      <c r="U1" s="4"/>
+      <c r="V1" s="4"/>
+      <c r="W1" s="4"/>
+      <c r="X1" s="4"/>
+      <c r="Y1" s="4"/>
+      <c r="Z1" s="4"/>
     </row>
     <row r="2" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="3" t="s">
+      <c r="A2" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C2" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="D2" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="E2" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="F2" s="3" t="s">
+      <c r="F2" s="5" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="3" t="s">
+      <c r="A3" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="B3" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="C3" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="D3" s="3" t="s">
+      <c r="D3" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="E3" s="3" t="s">
+      <c r="E3" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="F3" s="3" t="s">
+      <c r="F3" s="5" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="D4" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="E4" s="3" t="s">
+      <c r="E4" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="F4" s="3" t="s">
+      <c r="F4" s="5" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="3" t="s">
+      <c r="A5" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="B5" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="C5" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="D5" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="E5" s="3" t="s">
+      <c r="E5" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="F5" s="3" t="s">
+      <c r="F5" s="5" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="3" t="s">
+      <c r="A6" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="B6" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="C6" s="3" t="s">
+      <c r="C6" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="D6" s="3" t="s">
+      <c r="D6" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="E6" s="3" t="s">
+      <c r="E6" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="F6" s="3" t="s">
+      <c r="F6" s="5" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="3" t="s">
+      <c r="A7" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="B7" s="3" t="s">
+      <c r="B7" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="C7" s="3" t="s">
+      <c r="C7" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="D7" s="3" t="s">
+      <c r="D7" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="E7" s="3" t="s">
+      <c r="E7" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="F7" s="3" t="s">
+      <c r="F7" s="5" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="3" t="s">
+      <c r="A8" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="B8" s="3" t="s">
+      <c r="B8" s="5" t="s">
         <v>43</v>
       </c>
-      <c r="C8" s="3" t="s">
+      <c r="C8" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="D8" s="3" t="s">
+      <c r="D8" s="5" t="s">
         <v>45</v>
       </c>
-      <c r="E8" s="3" t="s">
+      <c r="E8" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="F8" s="3" t="s">
+      <c r="F8" s="5" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="3" t="s">
+      <c r="A9" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="B9" s="3" t="s">
+      <c r="B9" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="C9" s="3" t="s">
+      <c r="C9" s="5" t="s">
         <v>50</v>
       </c>
-      <c r="D9" s="3" t="s">
+      <c r="D9" s="5" t="s">
         <v>51</v>
       </c>
-      <c r="E9" s="3" t="s">
+      <c r="E9" s="5" t="s">
         <v>52</v>
       </c>
-      <c r="F9" s="3" t="s">
+      <c r="F9" s="5" t="s">
         <v>53</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="3" t="s">
+      <c r="A10" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="B10" s="3" t="s">
+      <c r="B10" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="C10" s="3" t="s">
+      <c r="C10" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="D10" s="3" t="s">
+      <c r="D10" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="E10" s="3" t="s">
+      <c r="E10" s="5" t="s">
         <v>58</v>
       </c>
-      <c r="F10" s="3" t="s">
+      <c r="F10" s="5" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="4" t="s">
+      <c r="A11" s="5" t="s">
         <v>60</v>
       </c>
-      <c r="B11" s="3" t="s">
+      <c r="B11" s="5" t="s">
         <v>61</v>
       </c>
-      <c r="C11" s="3" t="s">
+      <c r="C11" s="5" t="s">
         <v>62</v>
       </c>
-      <c r="D11" s="3" t="s">
+      <c r="D11" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="E11" s="3" t="s">
+      <c r="E11" s="5" t="s">
         <v>64</v>
       </c>
-      <c r="F11" s="3" t="s">
+      <c r="F11" s="5" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="3" t="s">
+      <c r="A12" s="5" t="s">
         <v>66</v>
       </c>
-      <c r="B12" s="3" t="s">
+      <c r="B12" s="5" t="s">
         <v>67</v>
       </c>
-      <c r="C12" s="3" t="s">
+      <c r="C12" s="5" t="s">
         <v>68</v>
       </c>
-      <c r="D12" s="3" t="s">
+      <c r="D12" s="5" t="s">
         <v>69</v>
       </c>
-      <c r="E12" s="3" t="s">
+      <c r="E12" s="5" t="s">
         <v>70</v>
       </c>
-      <c r="F12" s="3" t="s">
+      <c r="F12" s="5" t="s">
         <v>71</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="3" t="s">
+      <c r="A13" s="5" t="s">
         <v>72</v>
       </c>
-      <c r="B13" s="3" t="s">
+      <c r="B13" s="5" t="s">
         <v>73</v>
       </c>
-      <c r="C13" s="3" t="s">
+      <c r="C13" s="5" t="s">
         <v>74</v>
       </c>
-      <c r="D13" s="3" t="s">
+      <c r="D13" s="5" t="s">
         <v>75</v>
       </c>
-      <c r="E13" s="3" t="s">
+      <c r="E13" s="5" t="s">
         <v>76</v>
       </c>
-      <c r="F13" s="3" t="s">
+      <c r="F13" s="5" t="s">
         <v>77</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="3" t="s">
+      <c r="A14" s="5" t="s">
         <v>78</v>
       </c>
-      <c r="B14" s="3" t="s">
+      <c r="B14" s="5" t="s">
         <v>79</v>
       </c>
-      <c r="C14" s="3" t="s">
+      <c r="C14" s="5" t="s">
         <v>80</v>
       </c>
-      <c r="D14" s="3" t="s">
+      <c r="D14" s="5" t="s">
         <v>81</v>
       </c>
-      <c r="E14" s="3" t="s">
+      <c r="E14" s="5" t="s">
         <v>82</v>
       </c>
-      <c r="F14" s="3" t="s">
+      <c r="F14" s="5" t="s">
         <v>83</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="3" t="s">
+      <c r="A15" s="5" t="s">
         <v>84</v>
       </c>
-      <c r="B15" s="3" t="s">
+      <c r="B15" s="5" t="s">
         <v>85</v>
       </c>
-      <c r="C15" s="3" t="s">
+      <c r="C15" s="5" t="s">
         <v>86</v>
       </c>
-      <c r="D15" s="3" t="s">
+      <c r="D15" s="5" t="s">
         <v>87</v>
       </c>
-      <c r="E15" s="3" t="s">
+      <c r="E15" s="5" t="s">
         <v>88</v>
       </c>
-      <c r="F15" s="3" t="s">
+      <c r="F15" s="5" t="s">
         <v>89</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="3" t="s">
+      <c r="A16" s="5" t="s">
         <v>90</v>
       </c>
-      <c r="B16" s="3" t="s">
+      <c r="B16" s="5" t="s">
         <v>91</v>
       </c>
-      <c r="C16" s="3" t="s">
+      <c r="C16" s="5" t="s">
         <v>92</v>
       </c>
-      <c r="D16" s="3" t="s">
+      <c r="D16" s="5" t="s">
         <v>93</v>
       </c>
-      <c r="E16" s="3" t="s">
+      <c r="E16" s="5" t="s">
         <v>94</v>
       </c>
-      <c r="F16" s="3" t="s">
+      <c r="F16" s="5" t="s">
         <v>95</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="3" t="s">
+      <c r="A17" s="5" t="s">
         <v>96</v>
       </c>
-      <c r="B17" s="3" t="s">
+      <c r="B17" s="5" t="s">
         <v>97</v>
       </c>
-      <c r="C17" s="3" t="s">
+      <c r="C17" s="5" t="s">
         <v>98</v>
       </c>
-      <c r="D17" s="3" t="s">
+      <c r="D17" s="5" t="s">
         <v>99</v>
       </c>
-      <c r="E17" s="3" t="s">
+      <c r="E17" s="5" t="s">
         <v>100</v>
       </c>
-      <c r="F17" s="3" t="s">
+      <c r="F17" s="5" t="s">
         <v>101</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="3" t="s">
+      <c r="A18" s="5" t="s">
         <v>102</v>
       </c>
-      <c r="B18" s="3" t="s">
+      <c r="B18" s="5" t="s">
         <v>103</v>
       </c>
-      <c r="C18" s="3" t="s">
+      <c r="C18" s="5" t="s">
         <v>104</v>
       </c>
-      <c r="D18" s="3" t="s">
+      <c r="D18" s="5" t="s">
         <v>105</v>
       </c>
-      <c r="E18" s="3" t="s">
+      <c r="E18" s="5" t="s">
         <v>106</v>
       </c>
-      <c r="F18" s="3" t="s">
+      <c r="F18" s="5" t="s">
         <v>107</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="3" t="s">
+      <c r="A19" s="5" t="s">
         <v>108</v>
       </c>
-      <c r="B19" s="3" t="s">
+      <c r="B19" s="5" t="s">
         <v>109</v>
       </c>
-      <c r="C19" s="3" t="s">
+      <c r="C19" s="5" t="s">
         <v>110</v>
       </c>
-      <c r="D19" s="3" t="s">
+      <c r="D19" s="5" t="s">
         <v>111</v>
       </c>
-      <c r="E19" s="3" t="s">
+      <c r="E19" s="5" t="s">
         <v>112</v>
       </c>
-      <c r="F19" s="3" t="s">
+      <c r="F19" s="5" t="s">
         <v>113</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="4" t="s">
+      <c r="A20" s="5" t="s">
         <v>114</v>
       </c>
-      <c r="B20" s="3" t="s">
+      <c r="B20" s="5" t="s">
         <v>115</v>
       </c>
-      <c r="C20" s="3" t="s">
+      <c r="C20" s="5" t="s">
         <v>116</v>
       </c>
-      <c r="D20" s="3" t="s">
+      <c r="D20" s="5" t="s">
         <v>117</v>
       </c>
-      <c r="E20" s="3" t="s">
+      <c r="E20" s="5" t="s">
         <v>118</v>
       </c>
-      <c r="F20" s="3" t="s">
+      <c r="F20" s="5" t="s">
         <v>119</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="3" t="s">
+      <c r="A21" s="5" t="s">
         <v>120</v>
       </c>
-      <c r="B21" s="3" t="s">
+      <c r="B21" s="5" t="s">
         <v>121</v>
       </c>
-      <c r="C21" s="3" t="s">
+      <c r="C21" s="5" t="s">
         <v>122</v>
       </c>
-      <c r="D21" s="3" t="s">
+      <c r="D21" s="5" t="s">
         <v>123</v>
       </c>
-      <c r="E21" s="3" t="s">
+      <c r="E21" s="5" t="s">
         <v>124</v>
       </c>
-      <c r="F21" s="3" t="s">
+      <c r="F21" s="5" t="s">
         <v>125</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="3" t="s">
+      <c r="A22" s="5" t="s">
         <v>126</v>
       </c>
-      <c r="B22" s="3" t="s">
+      <c r="B22" s="5" t="s">
         <v>127</v>
       </c>
-      <c r="C22" s="3" t="s">
+      <c r="C22" s="5" t="s">
         <v>128</v>
       </c>
-      <c r="D22" s="3" t="s">
+      <c r="D22" s="5" t="s">
         <v>129</v>
       </c>
-      <c r="E22" s="3" t="s">
+      <c r="E22" s="5" t="s">
         <v>130</v>
       </c>
-      <c r="F22" s="3" t="s">
+      <c r="F22" s="5" t="s">
         <v>131</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="3" t="s">
+      <c r="A23" s="5" t="s">
         <v>132</v>
       </c>
-      <c r="B23" s="3" t="s">
+      <c r="B23" s="5" t="s">
         <v>133</v>
       </c>
-      <c r="C23" s="3" t="s">
+      <c r="C23" s="5" t="s">
         <v>134</v>
       </c>
-      <c r="D23" s="3" t="s">
+      <c r="D23" s="5" t="s">
         <v>135</v>
       </c>
-      <c r="E23" s="3" t="s">
+      <c r="E23" s="5" t="s">
         <v>136</v>
       </c>
-      <c r="F23" s="3" t="s">
+      <c r="F23" s="5" t="s">
         <v>137</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="3" t="s">
+      <c r="A24" s="5" t="s">
         <v>138</v>
       </c>
-      <c r="B24" s="3" t="s">
+      <c r="B24" s="5" t="s">
         <v>139</v>
       </c>
-      <c r="C24" s="3" t="s">
+      <c r="C24" s="5" t="s">
         <v>140</v>
       </c>
-      <c r="D24" s="3" t="s">
+      <c r="D24" s="5" t="s">
         <v>141</v>
       </c>
-      <c r="E24" s="3" t="s">
+      <c r="E24" s="5" t="s">
         <v>142</v>
       </c>
-      <c r="F24" s="3" t="s">
+      <c r="F24" s="5" t="s">
         <v>143</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="3" t="s">
+      <c r="A25" s="5" t="s">
         <v>144</v>
       </c>
-      <c r="B25" s="3" t="s">
+      <c r="B25" s="5" t="s">
         <v>145</v>
       </c>
-      <c r="C25" s="3" t="s">
+      <c r="C25" s="5" t="s">
         <v>146</v>
       </c>
-      <c r="D25" s="3" t="s">
+      <c r="D25" s="5" t="s">
         <v>147</v>
       </c>
-      <c r="E25" s="3" t="s">
+      <c r="E25" s="5" t="s">
         <v>148</v>
       </c>
-      <c r="F25" s="3" t="s">
+      <c r="F25" s="5" t="s">
         <v>149</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="3" t="s">
+      <c r="A26" s="5" t="s">
         <v>150</v>
       </c>
-      <c r="B26" s="3" t="s">
+      <c r="B26" s="5" t="s">
         <v>151</v>
       </c>
-      <c r="C26" s="3" t="s">
+      <c r="C26" s="5" t="s">
         <v>152</v>
       </c>
-      <c r="D26" s="3" t="s">
+      <c r="D26" s="5" t="s">
         <v>153</v>
       </c>
-      <c r="E26" s="3" t="s">
+      <c r="E26" s="5" t="s">
         <v>154</v>
       </c>
-      <c r="F26" s="3" t="s">
+      <c r="F26" s="5" t="s">
         <v>155</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="3" t="s">
+      <c r="A27" s="5" t="s">
         <v>156</v>
       </c>
-      <c r="B27" s="3" t="s">
+      <c r="B27" s="5" t="s">
         <v>157</v>
       </c>
-      <c r="C27" s="3" t="s">
+      <c r="C27" s="5" t="s">
         <v>158</v>
       </c>
-      <c r="D27" s="3" t="s">
+      <c r="D27" s="5" t="s">
         <v>159</v>
       </c>
-      <c r="E27" s="3" t="s">
+      <c r="E27" s="5" t="s">
         <v>160</v>
       </c>
-      <c r="F27" s="3" t="s">
+      <c r="F27" s="5" t="s">
         <v>161</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="3" t="s">
+      <c r="A28" s="5" t="s">
         <v>162</v>
       </c>
-      <c r="B28" s="3" t="s">
+      <c r="B28" s="5" t="s">
         <v>163</v>
       </c>
-      <c r="C28" s="3" t="s">
+      <c r="C28" s="5" t="s">
         <v>164</v>
       </c>
-      <c r="D28" s="3" t="s">
+      <c r="D28" s="5" t="s">
         <v>165</v>
       </c>
-      <c r="E28" s="3" t="s">
+      <c r="E28" s="5" t="s">
         <v>166</v>
       </c>
-      <c r="F28" s="3" t="s">
+      <c r="F28" s="5" t="s">
         <v>167</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="3" t="s">
+      <c r="A29" s="5" t="s">
         <v>168</v>
       </c>
-      <c r="B29" s="3" t="s">
+      <c r="B29" s="5" t="s">
         <v>169</v>
       </c>
-      <c r="C29" s="3" t="s">
+      <c r="C29" s="5" t="s">
         <v>170</v>
       </c>
-      <c r="D29" s="3" t="s">
+      <c r="D29" s="5" t="s">
         <v>171</v>
       </c>
-      <c r="E29" s="3" t="s">
+      <c r="E29" s="5" t="s">
         <v>172</v>
       </c>
-      <c r="F29" s="3" t="s">
+      <c r="F29" s="5" t="s">
         <v>173</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="4" t="s">
+      <c r="A30" s="5" t="s">
         <v>174</v>
       </c>
-      <c r="B30" s="3" t="s">
+      <c r="B30" s="5" t="s">
         <v>175</v>
       </c>
-      <c r="C30" s="3" t="s">
+      <c r="C30" s="5" t="s">
         <v>176</v>
       </c>
-      <c r="D30" s="3" t="s">
+      <c r="D30" s="5" t="s">
         <v>177</v>
       </c>
-      <c r="E30" s="3" t="s">
+      <c r="E30" s="5" t="s">
         <v>178</v>
       </c>
-      <c r="F30" s="3" t="s">
+      <c r="F30" s="5" t="s">
         <v>179</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="3" t="s">
+      <c r="A31" s="5" t="s">
         <v>180</v>
       </c>
-      <c r="B31" s="3" t="s">
+      <c r="B31" s="5" t="s">
         <v>181</v>
       </c>
-      <c r="C31" s="3" t="s">
+      <c r="C31" s="5" t="s">
         <v>182</v>
       </c>
-      <c r="D31" s="3" t="s">
+      <c r="D31" s="5" t="s">
         <v>183</v>
       </c>
-      <c r="E31" s="3" t="s">
+      <c r="E31" s="5" t="s">
         <v>184</v>
       </c>
-      <c r="F31" s="3" t="s">
+      <c r="F31" s="5" t="s">
         <v>185</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="3" t="s">
+      <c r="A32" s="5" t="s">
         <v>186</v>
       </c>
-      <c r="B32" s="3" t="s">
+      <c r="B32" s="5" t="s">
         <v>187</v>
       </c>
-      <c r="C32" s="3" t="s">
+      <c r="C32" s="5" t="s">
         <v>188</v>
       </c>
-      <c r="D32" s="3" t="s">
+      <c r="D32" s="5" t="s">
         <v>189</v>
       </c>
-      <c r="E32" s="3" t="s">
+      <c r="E32" s="5" t="s">
         <v>190</v>
       </c>
-      <c r="F32" s="3" t="s">
+      <c r="F32" s="5" t="s">
         <v>191</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="3" t="s">
+      <c r="A33" s="5" t="s">
         <v>192</v>
       </c>
-      <c r="B33" s="3" t="s">
+      <c r="B33" s="5" t="s">
         <v>193</v>
       </c>
-      <c r="C33" s="3" t="s">
+      <c r="C33" s="5" t="s">
         <v>194</v>
       </c>
-      <c r="D33" s="3" t="s">
+      <c r="D33" s="5" t="s">
         <v>195</v>
       </c>
-      <c r="E33" s="3" t="s">
+      <c r="E33" s="5" t="s">
         <v>196</v>
       </c>
-      <c r="F33" s="3" t="s">
+      <c r="F33" s="5" t="s">
         <v>197</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="3" t="s">
+      <c r="A34" s="5" t="s">
         <v>198</v>
       </c>
-      <c r="B34" s="3" t="s">
+      <c r="B34" s="5" t="s">
         <v>199</v>
       </c>
-      <c r="C34" s="3" t="s">
+      <c r="C34" s="5" t="s">
         <v>200</v>
       </c>
-      <c r="D34" s="3" t="s">
+      <c r="D34" s="5" t="s">
         <v>201</v>
       </c>
-      <c r="E34" s="3" t="s">
+      <c r="E34" s="5" t="s">
         <v>202</v>
       </c>
-      <c r="F34" s="3" t="s">
+      <c r="F34" s="5" t="s">
         <v>203</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="3" t="s">
+      <c r="A35" s="5" t="s">
         <v>204</v>
       </c>
-      <c r="B35" s="3" t="s">
+      <c r="B35" s="5" t="s">
         <v>205</v>
       </c>
-      <c r="C35" s="3" t="s">
+      <c r="C35" s="5" t="s">
         <v>206</v>
       </c>
-      <c r="D35" s="3" t="s">
+      <c r="D35" s="5" t="s">
         <v>207</v>
       </c>
-      <c r="E35" s="3" t="s">
+      <c r="E35" s="5" t="s">
         <v>208</v>
       </c>
-      <c r="F35" s="3" t="s">
+      <c r="F35" s="5" t="s">
         <v>209</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="3" t="s">
+      <c r="A36" s="5" t="s">
         <v>210</v>
       </c>
-      <c r="B36" s="3" t="s">
+      <c r="B36" s="5" t="s">
         <v>211</v>
       </c>
-      <c r="C36" s="3" t="s">
+      <c r="C36" s="5" t="s">
         <v>212</v>
       </c>
-      <c r="D36" s="3" t="s">
+      <c r="D36" s="5" t="s">
         <v>213</v>
       </c>
-      <c r="E36" s="3" t="s">
+      <c r="E36" s="5" t="s">
         <v>214</v>
       </c>
-      <c r="F36" s="3" t="s">
+      <c r="F36" s="5" t="s">
         <v>215</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="3" t="s">
+      <c r="A37" s="5" t="s">
         <v>216</v>
       </c>
-      <c r="B37" s="3" t="s">
+      <c r="B37" s="5" t="s">
         <v>217</v>
       </c>
-      <c r="C37" s="3" t="s">
+      <c r="C37" s="5" t="s">
         <v>218</v>
       </c>
-      <c r="D37" s="3" t="s">
+      <c r="D37" s="5" t="s">
         <v>219</v>
       </c>
-      <c r="E37" s="3" t="s">
+      <c r="E37" s="5" t="s">
         <v>220</v>
       </c>
-      <c r="F37" s="3" t="s">
+      <c r="F37" s="5" t="s">
         <v>221</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="3" t="s">
+      <c r="A38" s="5" t="s">
         <v>222</v>
       </c>
-      <c r="B38" s="3" t="s">
+      <c r="B38" s="5" t="s">
         <v>223</v>
       </c>
-      <c r="C38" s="3" t="s">
+      <c r="C38" s="5" t="s">
         <v>224</v>
       </c>
-      <c r="D38" s="3" t="s">
+      <c r="D38" s="5" t="s">
         <v>225</v>
       </c>
-      <c r="E38" s="3" t="s">
+      <c r="E38" s="5" t="s">
         <v>226</v>
       </c>
-      <c r="F38" s="3" t="s">
+      <c r="F38" s="5" t="s">
         <v>227</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="3" t="s">
+      <c r="A39" s="5" t="s">
         <v>228</v>
       </c>
-      <c r="B39" s="3" t="s">
+      <c r="B39" s="5" t="s">
         <v>229</v>
       </c>
-      <c r="C39" s="3" t="s">
+      <c r="C39" s="5" t="s">
         <v>230</v>
       </c>
-      <c r="D39" s="3" t="s">
+      <c r="D39" s="5" t="s">
         <v>231</v>
       </c>
-      <c r="E39" s="3" t="s">
+      <c r="E39" s="5" t="s">
         <v>232</v>
       </c>
-      <c r="F39" s="3" t="s">
+      <c r="F39" s="5" t="s">
         <v>233</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="4" t="s">
+      <c r="A40" s="5" t="s">
         <v>234</v>
       </c>
-      <c r="B40" s="3" t="s">
+      <c r="B40" s="5" t="s">
         <v>235</v>
       </c>
-      <c r="C40" s="3" t="s">
+      <c r="C40" s="5" t="s">
         <v>236</v>
       </c>
-      <c r="D40" s="3" t="s">
+      <c r="D40" s="5" t="s">
         <v>237</v>
       </c>
-      <c r="E40" s="3" t="s">
+      <c r="E40" s="5" t="s">
         <v>238</v>
       </c>
-      <c r="F40" s="3" t="s">
+      <c r="F40" s="5" t="s">
         <v>239</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="3" t="s">
+      <c r="A41" s="5" t="s">
         <v>240</v>
       </c>
-      <c r="B41" s="3" t="s">
+      <c r="B41" s="5" t="s">
         <v>241</v>
       </c>
-      <c r="C41" s="3" t="s">
+      <c r="C41" s="5" t="s">
         <v>242</v>
       </c>
-      <c r="D41" s="3" t="s">
+      <c r="D41" s="5" t="s">
         <v>243</v>
       </c>
-      <c r="E41" s="3" t="s">
+      <c r="E41" s="5" t="s">
         <v>244</v>
       </c>
-      <c r="F41" s="3" t="s">
+      <c r="F41" s="5" t="s">
         <v>245</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="3" t="s">
+      <c r="A42" s="5" t="s">
         <v>246</v>
       </c>
-      <c r="B42" s="3" t="s">
+      <c r="B42" s="5" t="s">
         <v>247</v>
       </c>
-      <c r="C42" s="3" t="s">
+      <c r="C42" s="5" t="s">
         <v>248</v>
       </c>
-      <c r="D42" s="3" t="s">
+      <c r="D42" s="5" t="s">
         <v>249</v>
       </c>
-      <c r="E42" s="3" t="s">
+      <c r="E42" s="5" t="s">
         <v>250</v>
       </c>
-      <c r="F42" s="3" t="s">
+      <c r="F42" s="5" t="s">
         <v>251</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="3" t="s">
+      <c r="A43" s="5" t="s">
         <v>252</v>
       </c>
-      <c r="B43" s="3" t="s">
+      <c r="B43" s="5" t="s">
         <v>253</v>
       </c>
-      <c r="C43" s="3" t="s">
+      <c r="C43" s="5" t="s">
         <v>254</v>
       </c>
-      <c r="D43" s="3" t="s">
+      <c r="D43" s="5" t="s">
         <v>255</v>
       </c>
-      <c r="E43" s="3" t="s">
+      <c r="E43" s="5" t="s">
         <v>256</v>
       </c>
-      <c r="F43" s="3" t="s">
+      <c r="F43" s="5" t="s">
         <v>257</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="3" t="s">
+      <c r="A44" s="5" t="s">
         <v>258</v>
       </c>
-      <c r="B44" s="3" t="s">
+      <c r="B44" s="5" t="s">
         <v>259</v>
       </c>
-      <c r="C44" s="3" t="s">
+      <c r="C44" s="5" t="s">
         <v>260</v>
       </c>
-      <c r="D44" s="3" t="s">
+      <c r="D44" s="5" t="s">
         <v>261</v>
       </c>
-      <c r="E44" s="3" t="s">
+      <c r="E44" s="5" t="s">
         <v>262</v>
       </c>
-      <c r="F44" s="3" t="s">
+      <c r="F44" s="5" t="s">
         <v>263</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="3" t="s">
+      <c r="A45" s="5" t="s">
         <v>264</v>
       </c>
-      <c r="B45" s="3" t="s">
+      <c r="B45" s="5" t="s">
         <v>265</v>
       </c>
-      <c r="C45" s="3" t="s">
+      <c r="C45" s="5" t="s">
         <v>266</v>
       </c>
-      <c r="D45" s="3" t="s">
+      <c r="D45" s="5" t="s">
         <v>267</v>
       </c>
-      <c r="E45" s="3" t="s">
+      <c r="E45" s="5" t="s">
         <v>268</v>
       </c>
-      <c r="F45" s="3" t="s">
+      <c r="F45" s="5" t="s">
         <v>269</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="3" t="s">
+      <c r="A46" s="5" t="s">
         <v>270</v>
       </c>
-      <c r="B46" s="3" t="s">
+      <c r="B46" s="5" t="s">
         <v>271</v>
       </c>
-      <c r="C46" s="3" t="s">
+      <c r="C46" s="5" t="s">
         <v>272</v>
       </c>
-      <c r="D46" s="3" t="s">
+      <c r="D46" s="5" t="s">
         <v>273</v>
       </c>
-      <c r="E46" s="3" t="s">
+      <c r="E46" s="5" t="s">
         <v>274</v>
       </c>
-      <c r="F46" s="3" t="s">
+      <c r="F46" s="5" t="s">
         <v>275</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A47" s="3" t="s">
+      <c r="A47" s="5" t="s">
         <v>276</v>
       </c>
-      <c r="B47" s="3" t="s">
+      <c r="B47" s="5" t="s">
         <v>277</v>
       </c>
-      <c r="C47" s="3" t="s">
+      <c r="C47" s="5" t="s">
         <v>278</v>
       </c>
-      <c r="D47" s="3" t="s">
+      <c r="D47" s="5" t="s">
         <v>279</v>
       </c>
-      <c r="E47" s="3" t="s">
+      <c r="E47" s="5" t="s">
         <v>280</v>
       </c>
-      <c r="F47" s="3" t="s">
+      <c r="F47" s="5" t="s">
         <v>281</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A48" s="3" t="s">
+      <c r="A48" s="5" t="s">
         <v>282</v>
       </c>
-      <c r="B48" s="3" t="s">
+      <c r="B48" s="5" t="s">
         <v>283</v>
       </c>
-      <c r="C48" s="3" t="s">
+      <c r="C48" s="5" t="s">
         <v>284</v>
       </c>
-      <c r="D48" s="3" t="s">
+      <c r="D48" s="5" t="s">
         <v>285</v>
       </c>
-      <c r="E48" s="3" t="s">
+      <c r="E48" s="5" t="s">
         <v>286</v>
       </c>
-      <c r="F48" s="3" t="s">
+      <c r="F48" s="5" t="s">
         <v>287</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A49" s="3" t="s">
+      <c r="A49" s="5" t="s">
         <v>288</v>
       </c>
-      <c r="B49" s="3" t="s">
+      <c r="B49" s="5" t="s">
         <v>278</v>
       </c>
-      <c r="C49" s="3" t="s">
+      <c r="C49" s="5" t="s">
         <v>278</v>
       </c>
-      <c r="D49" s="3" t="s">
+      <c r="D49" s="5" t="s">
         <v>289</v>
       </c>
-      <c r="E49" s="3" t="s">
+      <c r="E49" s="5" t="s">
         <v>290</v>
       </c>
-      <c r="F49" s="3" t="s">
+      <c r="F49" s="5" t="s">
         <v>291</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A50" s="3" t="s">
+      <c r="A50" s="5" t="s">
         <v>292</v>
       </c>
-      <c r="B50" s="3" t="s">
+      <c r="B50" s="5" t="s">
         <v>293</v>
       </c>
-      <c r="C50" s="3" t="s">
+      <c r="C50" s="5" t="s">
         <v>294</v>
       </c>
-      <c r="D50" s="3" t="s">
+      <c r="D50" s="5" t="s">
         <v>295</v>
       </c>
-      <c r="E50" s="3" t="s">
+      <c r="E50" s="5" t="s">
         <v>296</v>
       </c>
-      <c r="F50" s="3" t="s">
+      <c r="F50" s="5" t="s">
         <v>297</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A51" s="3" t="s">
+      <c r="A51" s="5" t="s">
         <v>298</v>
       </c>
-      <c r="B51" s="3" t="s">
+      <c r="B51" s="5" t="s">
         <v>299</v>
       </c>
-      <c r="C51" s="3" t="s">
+      <c r="C51" s="5" t="s">
         <v>300</v>
       </c>
-      <c r="D51" s="3" t="s">
+      <c r="D51" s="5" t="s">
         <v>301</v>
       </c>
-      <c r="E51" s="3" t="s">
+      <c r="E51" s="5" t="s">
         <v>302</v>
       </c>
-      <c r="F51" s="3" t="s">
+      <c r="F51" s="5" t="s">
         <v>303</v>
       </c>
     </row>

</xml_diff>